<commit_message>
Manning workbook: label windows and finish materials as client-paid, excluded from base
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NY6xq9eh2BK6Au4SE2w7Bc
</commit_message>
<xml_diff>
--- a/Manning_Bid_Leveling.xlsx
+++ b/Manning_Bid_Leveling.xlsx
@@ -99,6 +99,18 @@
         </r>
       </text>
     </comment>
+    <comment ref="B40" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Client budget for windows. Supply AND install are excluded from the contract (General Note 3). Window bids are tendered only so the client can order and we can lock the schedule.</t>
+        </r>
+      </text>
+    </comment>
     <comment ref="E5" authorId="0">
       <text>
         <r>
@@ -150,7 +162,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="177" uniqueCount="126">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="182" uniqueCount="131">
   <si>
     <t xml:space="preserve">439 Manning Ave: Base Scope Bid Leveling vs Budget and 35% Markup Target</t>
   </si>
@@ -290,7 +302,13 @@
     <t xml:space="preserve">Angled Skylight</t>
   </si>
   <si>
-    <t xml:space="preserve">Windows (client-paid, not in our cost)</t>
+    <t xml:space="preserve">Windows: CLIENT-PAID, NOT IN BASE COST (info only)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Finish materials: CLIENT-PAID, NOT IN BASE COST (hardwood, interior doors, hardware)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tender Package P9 budget; client selections</t>
   </si>
   <si>
     <t xml:space="preserve">Notes</t>
@@ -300,6 +318,15 @@
   </si>
   <si>
     <t xml:space="preserve">Contract sell $114,070 is the 2.0 Rear Addition base only (excludes design fees and add-ons), per the Tender Package margin check.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Base cost EXCLUDES windows (supply + install) and all client finish materials (hardwood, interior doors, hardware). Base includes only the install labour for hardwood, doors and trim inside General Works.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Confirm Renomar's and Fabiano's prices do NOT include supply of hardwood, interior doors or hardware, or window install. If they do, deduct it.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Safety Roofing combo includes the skylight (an add-on), so the base is slightly overstated when Safety is selected. That's conservative.</t>
   </si>
   <si>
     <t xml:space="preserve">Site Services has no quote yet; the $11,500 budget is carried at cost.</t>
@@ -1137,7 +1164,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:I46"/>
+  <dimension ref="A1:I50"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="40"/>
@@ -2055,10 +2082,16 @@
       <c r="I40" s="2"/>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A41" s="2"/>
-      <c r="B41" s="2"/>
+      <c r="A41" s="20" t="s">
+        <v>47</v>
+      </c>
+      <c r="B41" s="23" t="n">
+        <v>7549</v>
+      </c>
       <c r="C41" s="2"/>
-      <c r="D41" s="2"/>
+      <c r="D41" s="2" t="s">
+        <v>48</v>
+      </c>
       <c r="E41" s="2"/>
       <c r="F41" s="2"/>
       <c r="G41" s="2"/>
@@ -2066,9 +2099,7 @@
       <c r="I41" s="2"/>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A42" s="20" t="s">
-        <v>47</v>
-      </c>
+      <c r="A42" s="2"/>
       <c r="B42" s="2"/>
       <c r="C42" s="2"/>
       <c r="D42" s="2"/>
@@ -2079,8 +2110,8 @@
       <c r="I42" s="2"/>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A43" s="26" t="s">
-        <v>48</v>
+      <c r="A43" s="20" t="s">
+        <v>49</v>
       </c>
       <c r="B43" s="2"/>
       <c r="C43" s="2"/>
@@ -2093,7 +2124,7 @@
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="26" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="B44" s="2"/>
       <c r="C44" s="2"/>
@@ -2106,7 +2137,7 @@
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="26" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="B45" s="2"/>
       <c r="C45" s="2"/>
@@ -2119,7 +2150,7 @@
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="26" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="B46" s="2"/>
       <c r="C46" s="2"/>
@@ -2129,6 +2160,58 @@
       <c r="G46" s="2"/>
       <c r="H46" s="2"/>
       <c r="I46" s="2"/>
+    </row>
+    <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A47" s="26" t="s">
+        <v>53</v>
+      </c>
+      <c r="B47" s="2"/>
+      <c r="C47" s="2"/>
+      <c r="D47" s="2"/>
+      <c r="E47" s="2"/>
+      <c r="F47" s="2"/>
+      <c r="G47" s="2"/>
+      <c r="H47" s="2"/>
+      <c r="I47" s="2"/>
+    </row>
+    <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A48" s="26" t="s">
+        <v>54</v>
+      </c>
+      <c r="B48" s="2"/>
+      <c r="C48" s="2"/>
+      <c r="D48" s="2"/>
+      <c r="E48" s="2"/>
+      <c r="F48" s="2"/>
+      <c r="G48" s="2"/>
+      <c r="H48" s="2"/>
+      <c r="I48" s="2"/>
+    </row>
+    <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A49" s="26" t="s">
+        <v>55</v>
+      </c>
+      <c r="B49" s="2"/>
+      <c r="C49" s="2"/>
+      <c r="D49" s="2"/>
+      <c r="E49" s="2"/>
+      <c r="F49" s="2"/>
+      <c r="G49" s="2"/>
+      <c r="H49" s="2"/>
+      <c r="I49" s="2"/>
+    </row>
+    <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A50" s="26" t="s">
+        <v>56</v>
+      </c>
+      <c r="B50" s="2"/>
+      <c r="C50" s="2"/>
+      <c r="D50" s="2"/>
+      <c r="E50" s="2"/>
+      <c r="F50" s="2"/>
+      <c r="G50" s="2"/>
+      <c r="H50" s="2"/>
+      <c r="I50" s="2"/>
     </row>
   </sheetData>
   <conditionalFormatting sqref="G5:G15">
@@ -2183,14 +2266,14 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>52</v>
+        <v>57</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>53</v>
+        <v>58</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -2202,90 +2285,90 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="14" t="s">
-        <v>54</v>
+        <v>59</v>
       </c>
       <c r="B4" s="14" t="s">
-        <v>55</v>
+        <v>60</v>
       </c>
       <c r="C4" s="14" t="s">
-        <v>56</v>
+        <v>61</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="27" t="s">
-        <v>57</v>
+        <v>62</v>
       </c>
       <c r="B5" s="28" t="n">
         <v>114070</v>
       </c>
       <c r="C5" s="26" t="s">
-        <v>58</v>
+        <v>63</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="27" t="s">
-        <v>59</v>
+        <v>64</v>
       </c>
       <c r="B6" s="29" t="n">
         <v>0.35</v>
       </c>
       <c r="C6" s="26" t="s">
-        <v>60</v>
+        <v>65</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="27" t="s">
-        <v>61</v>
+        <v>66</v>
       </c>
       <c r="B7" s="28" t="n">
         <v>20000</v>
       </c>
       <c r="C7" s="26" t="s">
-        <v>62</v>
+        <v>67</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="27" t="s">
-        <v>63</v>
+        <v>68</v>
       </c>
       <c r="B8" s="30" t="s">
-        <v>64</v>
+        <v>69</v>
       </c>
       <c r="C8" s="26" t="s">
-        <v>65</v>
+        <v>70</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="27" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="B9" s="28" t="n">
         <v>6290</v>
       </c>
       <c r="C9" s="26" t="s">
-        <v>67</v>
+        <v>72</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="27" t="s">
-        <v>68</v>
+        <v>73</v>
       </c>
       <c r="B10" s="30" t="s">
-        <v>69</v>
+        <v>74</v>
       </c>
       <c r="C10" s="26" t="s">
-        <v>70</v>
+        <v>75</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="27" t="s">
-        <v>71</v>
+        <v>76</v>
       </c>
       <c r="B11" s="29" t="n">
         <v>0.1</v>
       </c>
       <c r="C11" s="26" t="s">
-        <v>72</v>
+        <v>77</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2296,7 +2379,7 @@
         <v>5000</v>
       </c>
       <c r="C12" s="26" t="s">
-        <v>73</v>
+        <v>78</v>
       </c>
     </row>
   </sheetData>
@@ -2337,7 +2420,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>74</v>
+        <v>79</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
@@ -2347,7 +2430,7 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>75</v>
+        <v>80</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -2368,30 +2451,30 @@
         <v>1</v>
       </c>
       <c r="B4" s="22" t="s">
-        <v>76</v>
+        <v>81</v>
       </c>
       <c r="C4" s="22" t="s">
-        <v>77</v>
+        <v>82</v>
       </c>
       <c r="D4" s="22" t="s">
-        <v>78</v>
+        <v>83</v>
       </c>
       <c r="E4" s="22" t="s">
-        <v>79</v>
+        <v>84</v>
       </c>
       <c r="F4" s="22" t="s">
-        <v>80</v>
+        <v>85</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="31" t="s">
-        <v>81</v>
+        <v>86</v>
       </c>
       <c r="B5" s="31" t="s">
-        <v>82</v>
+        <v>87</v>
       </c>
       <c r="C5" s="31" t="s">
-        <v>83</v>
+        <v>88</v>
       </c>
       <c r="D5" s="6" t="n">
         <v>57100</v>
@@ -2406,13 +2489,13 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="31" t="s">
-        <v>81</v>
+        <v>86</v>
       </c>
       <c r="B6" s="31" t="s">
-        <v>84</v>
+        <v>89</v>
       </c>
       <c r="C6" s="31" t="s">
-        <v>85</v>
+        <v>90</v>
       </c>
       <c r="D6" s="6" t="n">
         <v>0</v>
@@ -2427,13 +2510,13 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="31" t="s">
-        <v>86</v>
+        <v>91</v>
       </c>
       <c r="B7" s="31" t="s">
-        <v>87</v>
+        <v>92</v>
       </c>
       <c r="C7" s="31" t="s">
-        <v>85</v>
+        <v>90</v>
       </c>
       <c r="D7" s="6" t="n">
         <v>0</v>
@@ -2448,13 +2531,13 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="31" t="s">
-        <v>86</v>
+        <v>91</v>
       </c>
       <c r="B8" s="31" t="s">
-        <v>88</v>
+        <v>93</v>
       </c>
       <c r="C8" s="31" t="s">
-        <v>89</v>
+        <v>94</v>
       </c>
       <c r="D8" s="6" t="n">
         <v>0</v>
@@ -2469,13 +2552,13 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="31" t="s">
-        <v>86</v>
+        <v>91</v>
       </c>
       <c r="B9" s="31" t="s">
-        <v>90</v>
+        <v>95</v>
       </c>
       <c r="C9" s="31" t="s">
-        <v>89</v>
+        <v>94</v>
       </c>
       <c r="D9" s="6" t="n">
         <v>0</v>
@@ -2490,13 +2573,13 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="31" t="s">
-        <v>91</v>
+        <v>96</v>
       </c>
       <c r="B10" s="31" t="s">
-        <v>92</v>
+        <v>97</v>
       </c>
       <c r="C10" s="31" t="s">
-        <v>83</v>
+        <v>88</v>
       </c>
       <c r="D10" s="6" t="n">
         <v>14000</v>
@@ -2511,13 +2594,13 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="31" t="s">
-        <v>91</v>
+        <v>96</v>
       </c>
       <c r="B11" s="31" t="s">
-        <v>93</v>
+        <v>98</v>
       </c>
       <c r="C11" s="31" t="s">
-        <v>85</v>
+        <v>90</v>
       </c>
       <c r="D11" s="6" t="n">
         <v>0</v>
@@ -2532,13 +2615,13 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="31" t="s">
-        <v>91</v>
+        <v>96</v>
       </c>
       <c r="B12" s="31" t="s">
+        <v>99</v>
+      </c>
+      <c r="C12" s="31" t="s">
         <v>94</v>
-      </c>
-      <c r="C12" s="31" t="s">
-        <v>89</v>
       </c>
       <c r="D12" s="6" t="n">
         <v>0</v>
@@ -2553,13 +2636,13 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="31" t="s">
-        <v>95</v>
+        <v>100</v>
       </c>
       <c r="B13" s="31" t="s">
-        <v>96</v>
+        <v>101</v>
       </c>
       <c r="C13" s="31" t="s">
-        <v>83</v>
+        <v>88</v>
       </c>
       <c r="D13" s="6" t="n">
         <v>6386.19</v>
@@ -2574,13 +2657,13 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="31" t="s">
-        <v>95</v>
+        <v>100</v>
       </c>
       <c r="B14" s="31" t="s">
-        <v>97</v>
+        <v>102</v>
       </c>
       <c r="C14" s="31" t="s">
-        <v>83</v>
+        <v>88</v>
       </c>
       <c r="D14" s="6" t="n">
         <v>7040</v>
@@ -2595,13 +2678,13 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="31" t="s">
-        <v>95</v>
+        <v>100</v>
       </c>
       <c r="B15" s="31" t="s">
-        <v>98</v>
+        <v>103</v>
       </c>
       <c r="C15" s="31" t="s">
-        <v>83</v>
+        <v>88</v>
       </c>
       <c r="D15" s="6" t="n">
         <v>7208.9</v>
@@ -2619,10 +2702,10 @@
         <v>14</v>
       </c>
       <c r="B16" s="31" t="s">
-        <v>99</v>
+        <v>104</v>
       </c>
       <c r="C16" s="31" t="s">
-        <v>83</v>
+        <v>88</v>
       </c>
       <c r="D16" s="6" t="n">
         <v>15700</v>
@@ -2640,10 +2723,10 @@
         <v>14</v>
       </c>
       <c r="B17" s="31" t="s">
-        <v>100</v>
+        <v>105</v>
       </c>
       <c r="C17" s="31" t="s">
-        <v>89</v>
+        <v>94</v>
       </c>
       <c r="D17" s="6" t="n">
         <v>0</v>
@@ -2661,10 +2744,10 @@
         <v>14</v>
       </c>
       <c r="B18" s="31" t="s">
-        <v>101</v>
+        <v>106</v>
       </c>
       <c r="C18" s="31" t="s">
-        <v>89</v>
+        <v>94</v>
       </c>
       <c r="D18" s="6" t="n">
         <v>0</v>
@@ -2679,13 +2762,13 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="31" t="s">
-        <v>102</v>
+        <v>107</v>
       </c>
       <c r="B19" s="31" t="s">
-        <v>103</v>
+        <v>108</v>
       </c>
       <c r="C19" s="31" t="s">
-        <v>83</v>
+        <v>88</v>
       </c>
       <c r="D19" s="6" t="n">
         <v>7900</v>
@@ -2700,13 +2783,13 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="31" t="s">
-        <v>102</v>
+        <v>107</v>
       </c>
       <c r="B20" s="31" t="s">
-        <v>104</v>
+        <v>109</v>
       </c>
       <c r="C20" s="31" t="s">
-        <v>89</v>
+        <v>94</v>
       </c>
       <c r="D20" s="6" t="n">
         <v>0</v>
@@ -2721,13 +2804,13 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="31" t="s">
-        <v>105</v>
+        <v>110</v>
       </c>
       <c r="B21" s="31" t="s">
-        <v>106</v>
+        <v>111</v>
       </c>
       <c r="C21" s="31" t="s">
-        <v>83</v>
+        <v>88</v>
       </c>
       <c r="D21" s="6" t="n">
         <v>20580</v>
@@ -2742,13 +2825,13 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="31" t="s">
-        <v>107</v>
+        <v>112</v>
       </c>
       <c r="B22" s="31" t="s">
-        <v>108</v>
+        <v>113</v>
       </c>
       <c r="C22" s="31" t="s">
-        <v>83</v>
+        <v>88</v>
       </c>
       <c r="D22" s="6" t="n">
         <v>9370</v>
@@ -2763,13 +2846,13 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="31" t="s">
-        <v>107</v>
+        <v>112</v>
       </c>
       <c r="B23" s="31" t="s">
-        <v>109</v>
+        <v>114</v>
       </c>
       <c r="C23" s="31" t="s">
-        <v>83</v>
+        <v>88</v>
       </c>
       <c r="D23" s="6" t="n">
         <v>9950</v>
@@ -2784,13 +2867,13 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="31" t="s">
-        <v>107</v>
+        <v>112</v>
       </c>
       <c r="B24" s="31" t="s">
-        <v>110</v>
+        <v>115</v>
       </c>
       <c r="C24" s="31" t="s">
-        <v>89</v>
+        <v>94</v>
       </c>
       <c r="D24" s="6" t="n">
         <v>0</v>
@@ -2805,13 +2888,13 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="31" t="s">
-        <v>107</v>
+        <v>112</v>
       </c>
       <c r="B25" s="31" t="s">
-        <v>111</v>
+        <v>116</v>
       </c>
       <c r="C25" s="31" t="s">
-        <v>89</v>
+        <v>94</v>
       </c>
       <c r="D25" s="6" t="n">
         <v>0</v>
@@ -2829,10 +2912,10 @@
         <v>18</v>
       </c>
       <c r="B26" s="31" t="s">
-        <v>112</v>
+        <v>117</v>
       </c>
       <c r="C26" s="31" t="s">
-        <v>83</v>
+        <v>88</v>
       </c>
       <c r="D26" s="6" t="n">
         <v>3360.5</v>
@@ -2847,13 +2930,13 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="31" t="s">
-        <v>113</v>
+        <v>118</v>
       </c>
       <c r="B27" s="31" t="s">
-        <v>114</v>
+        <v>119</v>
       </c>
       <c r="C27" s="31" t="s">
-        <v>83</v>
+        <v>88</v>
       </c>
       <c r="D27" s="6" t="n">
         <v>7850</v>
@@ -2868,13 +2951,13 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="31" t="s">
-        <v>113</v>
+        <v>118</v>
       </c>
       <c r="B28" s="31" t="s">
-        <v>115</v>
+        <v>120</v>
       </c>
       <c r="C28" s="31" t="s">
-        <v>83</v>
+        <v>88</v>
       </c>
       <c r="D28" s="6" t="n">
         <v>8340</v>
@@ -2889,13 +2972,13 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="31" t="s">
-        <v>113</v>
+        <v>118</v>
       </c>
       <c r="B29" s="31" t="s">
-        <v>116</v>
+        <v>121</v>
       </c>
       <c r="C29" s="31" t="s">
-        <v>83</v>
+        <v>88</v>
       </c>
       <c r="D29" s="6" t="n">
         <v>9646.02</v>
@@ -2910,13 +2993,13 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="31" t="s">
-        <v>117</v>
+        <v>122</v>
       </c>
       <c r="B30" s="31" t="s">
-        <v>118</v>
+        <v>123</v>
       </c>
       <c r="C30" s="31" t="s">
-        <v>83</v>
+        <v>88</v>
       </c>
       <c r="D30" s="6" t="n">
         <v>31200</v>
@@ -2931,13 +3014,13 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="31" t="s">
-        <v>119</v>
+        <v>124</v>
       </c>
       <c r="B31" s="31" t="s">
-        <v>118</v>
+        <v>123</v>
       </c>
       <c r="C31" s="31" t="s">
-        <v>83</v>
+        <v>88</v>
       </c>
       <c r="D31" s="6" t="n">
         <v>10800</v>
@@ -2952,13 +3035,13 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="31" t="s">
-        <v>120</v>
+        <v>125</v>
       </c>
       <c r="B32" s="31" t="s">
-        <v>121</v>
+        <v>126</v>
       </c>
       <c r="C32" s="31" t="s">
-        <v>83</v>
+        <v>88</v>
       </c>
       <c r="D32" s="6" t="n">
         <v>3300</v>
@@ -2973,13 +3056,13 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="31" t="s">
-        <v>120</v>
+        <v>125</v>
       </c>
       <c r="B33" s="31" t="s">
-        <v>122</v>
+        <v>127</v>
       </c>
       <c r="C33" s="31" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="D33" s="6" t="n">
         <v>300</v>
@@ -2994,13 +3077,13 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="31" t="s">
-        <v>124</v>
+        <v>129</v>
       </c>
       <c r="B34" s="31" t="s">
-        <v>125</v>
+        <v>130</v>
       </c>
       <c r="C34" s="31" t="s">
-        <v>83</v>
+        <v>88</v>
       </c>
       <c r="D34" s="6" t="n">
         <v>1215</v>

</xml_diff>